<commit_message>
Updated POL_grids_kan50 model - 2026-09-05 02:00
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_POL_grids_kan50/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6886E1BB-D2D6-4A9C-AC34-BA4334CB1883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1593261B-018E-42A2-8374-FD8809C3FAAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -711,196 +711,244 @@
     <t>pre</t>
   </si>
   <si>
+    <t>distr_solelc_spv_POL_005</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 5</t>
+  </si>
+  <si>
+    <t>NRGI</t>
+  </si>
+  <si>
+    <t>daynite</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_006</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 6</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_010</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 10</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_002</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 2</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_019</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 19</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_009</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 9</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_017</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 17</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_020</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 20</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_014</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 14</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_013</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 13</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_001</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 1</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_015</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 15</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_018</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 18</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_003</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 3</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_007</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 7</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_016</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 16</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_004</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 4</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_012</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 12</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_011</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 11</t>
+  </si>
+  <si>
     <t>distr_solelc_spv_POL_008</t>
   </si>
   <si>
     <t>connecting solar to buses in cluster 8</t>
   </si>
   <si>
-    <t>NRGI</t>
-  </si>
-  <si>
-    <t>daynite</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_013</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 13</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_004</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 4</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_002</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 2</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_019</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 19</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_009</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 9</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_012</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 12</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_011</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 11</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_003</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 3</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_007</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 7</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_016</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 16</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_006</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 6</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_010</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 10</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_001</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 1</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_015</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 15</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_018</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 18</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_005</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 5</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_014</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 14</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_017</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 17</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_020</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 20</t>
-  </si>
-  <si>
     <t>comm-in</t>
   </si>
   <si>
     <t>ncap_cost~USD21_alt</t>
   </si>
   <si>
+    <t>e_Lubin_POL,e_Poznan_POL,e_Koszalin_POL,e_Bydgoszcz_POL</t>
+  </si>
+  <si>
+    <t>e_Plock_POL,e_Olsztyn_POL,e_Warsaw_POL</t>
+  </si>
+  <si>
+    <t>e_Elk_POL,e_Grajewo_POL</t>
+  </si>
+  <si>
+    <t>e_Legnica_POL,e_Swidnica_POL,e_KedzierzynKozle_POL,e_Opole_POL</t>
+  </si>
+  <si>
+    <t>e_Kielce_POL,e_Warsaw_POL,e_OstrowiecSwietokrz_POL</t>
+  </si>
+  <si>
+    <t>e_Pulawy_POL,e_Bialystok_POL,e_Chelm_POL</t>
+  </si>
+  <si>
+    <t>e_Konin_POL,e_Bydgoszcz_POL,e_Wloclawek_POL,e_Kwidzyn_POL,e_Plock_POL</t>
+  </si>
+  <si>
+    <t>e_OstrowiecSwietokrz_POL,e_Pulawy_POL,e_Warsaw_POL</t>
+  </si>
+  <si>
+    <t>e_BielskoBiala_POL,e_Katowice_POL,e_Krakow_POL,e_Tarnow_POL</t>
+  </si>
+  <si>
+    <t>e_Rzeszow_POL,e_Zamosc_POL,e_Pulawy_POL,e_Chelm_POL</t>
+  </si>
+  <si>
+    <t>e_Boleslawiec_POL,e_ZielonaGora_POL</t>
+  </si>
+  <si>
+    <t>e_Sosnowiec_POL,e_KedzierzynKozle_POL,e_Olesnica_POL,e_Gliwice_POL,e_Czestochowa_POL,e_Radomsko_POL,e_PiotrkowTrybunalsk_POL,e_Kielce_POL</t>
+  </si>
+  <si>
+    <t>e_Warsaw_POL,e_Lomza_POL</t>
+  </si>
+  <si>
+    <t>e_Lubin_POL,e_Swidnica_POL,e_Wroclaw_POL,e_Poznan_POL,e_Olesnica_POL</t>
+  </si>
+  <si>
+    <t>e_Koszalin_POL,e_Ustka_POL,e_Slupsk_POL</t>
+  </si>
+  <si>
+    <t>e_Olesnica_POL,e_Konin_POL,e_PiotrkowTrybunalsk_POL,e_Plock_POL</t>
+  </si>
+  <si>
+    <t>e_GorzowWielkopolski_POL,e_Szczecin_POL,e_Police_POL</t>
+  </si>
+  <si>
+    <t>e_Krosno_POL,e_Mielec_POL,e_Debica_POL,e_Zamosc_POL</t>
+  </si>
+  <si>
+    <t>e_Lomza_POL,e_Elk_POL,e_Bialystok_POL,e_Grajewo_POL</t>
+  </si>
+  <si>
     <t>e_Bydgoszcz_POL,e_Gdansk_POL,e_Grudziadz_POL,e_Kwidzyn_POL</t>
   </si>
   <si>
-    <t>e_Rzeszow_POL,e_Zamosc_POL,e_Pulawy_POL,e_Chelm_POL</t>
-  </si>
-  <si>
-    <t>e_GorzowWielkopolski_POL,e_Szczecin_POL,e_Police_POL</t>
-  </si>
-  <si>
-    <t>e_Legnica_POL,e_Swidnica_POL,e_KedzierzynKozle_POL,e_Opole_POL</t>
-  </si>
-  <si>
-    <t>e_Kielce_POL,e_Warsaw_POL,e_OstrowiecSwietokrz_POL</t>
-  </si>
-  <si>
-    <t>e_Pulawy_POL,e_Bialystok_POL,e_Chelm_POL</t>
-  </si>
-  <si>
-    <t>e_Krosno_POL,e_Mielec_POL,e_Debica_POL,e_Zamosc_POL</t>
-  </si>
-  <si>
-    <t>e_Lomza_POL,e_Elk_POL,e_Bialystok_POL,e_Grajewo_POL</t>
-  </si>
-  <si>
-    <t>e_Lubin_POL,e_Swidnica_POL,e_Wroclaw_POL,e_Poznan_POL,e_Olesnica_POL</t>
-  </si>
-  <si>
-    <t>e_Koszalin_POL,e_Ustka_POL,e_Slupsk_POL</t>
-  </si>
-  <si>
-    <t>e_Olesnica_POL,e_Konin_POL,e_PiotrkowTrybunalsk_POL,e_Plock_POL</t>
-  </si>
-  <si>
-    <t>e_Plock_POL,e_Olsztyn_POL,e_Warsaw_POL</t>
-  </si>
-  <si>
-    <t>e_Elk_POL,e_Grajewo_POL</t>
-  </si>
-  <si>
-    <t>e_Boleslawiec_POL,e_ZielonaGora_POL</t>
-  </si>
-  <si>
-    <t>e_Sosnowiec_POL,e_KedzierzynKozle_POL,e_Olesnica_POL,e_Gliwice_POL,e_Czestochowa_POL,e_Radomsko_POL,e_PiotrkowTrybunalsk_POL,e_Kielce_POL</t>
-  </si>
-  <si>
-    <t>e_Warsaw_POL,e_Lomza_POL</t>
-  </si>
-  <si>
-    <t>e_Lubin_POL,e_Poznan_POL,e_Koszalin_POL,e_Bydgoszcz_POL</t>
-  </si>
-  <si>
-    <t>e_BielskoBiala_POL,e_Katowice_POL,e_Krakow_POL,e_Tarnow_POL</t>
-  </si>
-  <si>
-    <t>e_Konin_POL,e_Bydgoszcz_POL,e_Wloclawek_POL,e_Kwidzyn_POL,e_Plock_POL</t>
-  </si>
-  <si>
-    <t>e_OstrowiecSwietokrz_POL,e_Pulawy_POL,e_Warsaw_POL</t>
+    <t>distr_wonelc_won_POL_014</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 14</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_020</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 20</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_018</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 18</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_006</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 6</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_009</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 9</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_004</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 4</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_012</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 12</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_003</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 3</t>
   </si>
   <si>
     <t>distr_wonelc_won_POL_019</t>
@@ -921,42 +969,24 @@
     <t>connecting wind onshore to buses in cluster 7</t>
   </si>
   <si>
+    <t>distr_wonelc_won_POL_011</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 11</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_010</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 10</t>
+  </si>
+  <si>
     <t>distr_wonelc_won_POL_005</t>
   </si>
   <si>
     <t>connecting wind onshore to buses in cluster 5</t>
   </si>
   <si>
-    <t>distr_wonelc_won_POL_018</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 18</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_011</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 11</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_010</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 10</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_012</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 12</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_003</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 3</t>
-  </si>
-  <si>
     <t>distr_wonelc_won_POL_002</t>
   </si>
   <si>
@@ -987,42 +1017,57 @@
     <t>connecting wind onshore to buses in cluster 8</t>
   </si>
   <si>
-    <t>distr_wonelc_won_POL_014</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 14</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_020</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 20</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_006</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 6</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_009</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 9</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_004</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 4</t>
-  </si>
-  <si>
     <t>distr_wonelc_won_POL_001</t>
   </si>
   <si>
     <t>connecting wind onshore to buses in cluster 1</t>
   </si>
   <si>
+    <t>elc_won_POL_014</t>
+  </si>
+  <si>
+    <t>e_Lubin_POL,e_Poznan_POL,e_Bydgoszcz_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_020</t>
+  </si>
+  <si>
+    <t>e_Sosnowiec_POL,e_KedzierzynKozle_POL,e_Olesnica_POL,e_Gliwice_POL,e_Czestochowa_POL,e_Radomsko_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_018</t>
+  </si>
+  <si>
+    <t>e_Boleslawiec_POL,e_Legnica_POL,e_Swidnica_POL,e_KedzierzynKozle_POL,e_Opole_POL,e_Olesnica_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_006</t>
+  </si>
+  <si>
+    <t>e_Olesnica_POL,e_Konin_POL,e_Bydgoszcz_POL,e_Wloclawek_POL,e_Kwidzyn_POL,e_Plock_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_009</t>
+  </si>
+  <si>
+    <t>e_Gdansk_POL,e_Grudziadz_POL,e_Kwidzyn_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_004</t>
+  </si>
+  <si>
+    <t>elc_won_POL_012</t>
+  </si>
+  <si>
+    <t>e_ZielonaGora_POL,e_GorzowWielkopolski_POL,e_Szczecin_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_003</t>
+  </si>
+  <si>
+    <t>e_Warsaw_POL,e_Lomza_POL,e_Pulawy_POL,e_Bialystok_POL</t>
+  </si>
+  <si>
     <t>elc_won_POL_019</t>
   </si>
   <si>
@@ -1041,42 +1086,24 @@
     <t>e_Warsaw_POL,e_Plock_POL,e_Olsztyn_POL</t>
   </si>
   <si>
+    <t>elc_won_POL_011</t>
+  </si>
+  <si>
+    <t>e_Boleslawiec_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_010</t>
+  </si>
+  <si>
+    <t>e_Police_POL,e_Koszalin_POL,e_Poznan_POL,e_Ustka_POL,e_Bydgoszcz_POL,e_Slupsk_POL,e_Gdansk_POL</t>
+  </si>
+  <si>
     <t>elc_won_POL_005</t>
   </si>
   <si>
     <t>e_Lomza_POL,e_Elk_POL,e_Grajewo_POL,e_Bialystok_POL,e_Chelm_POL</t>
   </si>
   <si>
-    <t>elc_won_POL_018</t>
-  </si>
-  <si>
-    <t>e_Boleslawiec_POL,e_Legnica_POL,e_Swidnica_POL,e_KedzierzynKozle_POL,e_Opole_POL,e_Olesnica_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_011</t>
-  </si>
-  <si>
-    <t>e_Boleslawiec_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_010</t>
-  </si>
-  <si>
-    <t>e_Police_POL,e_Koszalin_POL,e_Poznan_POL,e_Ustka_POL,e_Bydgoszcz_POL,e_Slupsk_POL,e_Gdansk_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_012</t>
-  </si>
-  <si>
-    <t>e_ZielonaGora_POL,e_GorzowWielkopolski_POL,e_Szczecin_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_003</t>
-  </si>
-  <si>
-    <t>e_Warsaw_POL,e_Lomza_POL,e_Pulawy_POL,e_Bialystok_POL</t>
-  </si>
-  <si>
     <t>elc_won_POL_002</t>
   </si>
   <si>
@@ -1107,33 +1134,6 @@
     <t>e_Olsztyn_POL,e_Elk_POL</t>
   </si>
   <si>
-    <t>elc_won_POL_014</t>
-  </si>
-  <si>
-    <t>e_Lubin_POL,e_Poznan_POL,e_Bydgoszcz_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_020</t>
-  </si>
-  <si>
-    <t>e_Sosnowiec_POL,e_KedzierzynKozle_POL,e_Olesnica_POL,e_Gliwice_POL,e_Czestochowa_POL,e_Radomsko_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_006</t>
-  </si>
-  <si>
-    <t>e_Olesnica_POL,e_Konin_POL,e_Bydgoszcz_POL,e_Wloclawek_POL,e_Kwidzyn_POL,e_Plock_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_009</t>
-  </si>
-  <si>
-    <t>e_Gdansk_POL,e_Grudziadz_POL,e_Kwidzyn_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_004</t>
-  </si>
-  <si>
     <t>elc_won_POL_001</t>
   </si>
   <si>
@@ -1152,34 +1152,46 @@
     <t>connecting wind offshore to buses in cluster 7</t>
   </si>
   <si>
+    <t>distr_wofelc_wof_POL_010</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 10</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_POL_009</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 9</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_POL_004</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 4</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_POL_006</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 6</t>
+  </si>
+  <si>
     <t>distr_wofelc_wof_POL_002</t>
   </si>
   <si>
     <t>connecting wind offshore to buses in cluster 2</t>
   </si>
   <si>
-    <t>distr_wofelc_wof_POL_006</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 6</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_POL_004</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 4</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_POL_010</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 10</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_POL_009</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 9</t>
+    <t>distr_wofelc_wof_POL_005</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 5</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_POL_001</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 1</t>
   </si>
   <si>
     <t>distr_wofelc_wof_POL_003</t>
@@ -1188,18 +1200,6 @@
     <t>connecting wind offshore to buses in cluster 3</t>
   </si>
   <si>
-    <t>distr_wofelc_wof_POL_005</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 5</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_POL_001</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 1</t>
-  </si>
-  <si>
     <t>elc_wof_POL_008</t>
   </si>
   <si>
@@ -1212,43 +1212,43 @@
     <t>e_Koszalin_POL</t>
   </si>
   <si>
+    <t>elc_wof_POL_010</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_009</t>
+  </si>
+  <si>
+    <t>e_Koszalin_POL,e_Ustka_POL</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_004</t>
+  </si>
+  <si>
+    <t>e_Ustka_POL,e_Gdynia_POL</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_006</t>
+  </si>
+  <si>
+    <t>e_Gdynia_POL</t>
+  </si>
+  <si>
     <t>elc_wof_POL_002</t>
   </si>
   <si>
     <t>e_Gdynia_POL,e_Gdansk_POL</t>
   </si>
   <si>
-    <t>elc_wof_POL_006</t>
-  </si>
-  <si>
-    <t>e_Gdynia_POL</t>
-  </si>
-  <si>
-    <t>elc_wof_POL_004</t>
-  </si>
-  <si>
-    <t>e_Ustka_POL,e_Gdynia_POL</t>
-  </si>
-  <si>
-    <t>elc_wof_POL_010</t>
-  </si>
-  <si>
-    <t>elc_wof_POL_009</t>
-  </si>
-  <si>
-    <t>e_Koszalin_POL,e_Ustka_POL</t>
+    <t>elc_wof_POL_005</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_001</t>
+  </si>
+  <si>
+    <t>e_Gdansk_POL</t>
   </si>
   <si>
     <t>elc_wof_POL_003</t>
-  </si>
-  <si>
-    <t>e_Gdansk_POL</t>
-  </si>
-  <si>
-    <t>elc_wof_POL_005</t>
-  </si>
-  <si>
-    <t>elc_wof_POL_001</t>
   </si>
   <si>
     <t>e_won_POL_001</t>
@@ -5844,7 +5844,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02F0484B-22D0-4E0E-A716-2E666EF2C9D0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0C0ECA9-2976-4949-BB23-4E467F422200}">
   <dimension ref="B9:BD30"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6082,16 +6082,16 @@
         <v>215</v>
       </c>
       <c r="Y11" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="Z11" t="s">
         <v>259</v>
       </c>
       <c r="AA11">
-        <v>0.99693515631487983</v>
+        <v>0.99730738889353909</v>
       </c>
       <c r="AB11">
-        <v>56.188800893869058</v>
+        <v>49.364536951784054</v>
       </c>
       <c r="AD11" t="s">
         <v>214</v>
@@ -6124,10 +6124,10 @@
         <v>320</v>
       </c>
       <c r="AO11">
-        <v>0.99872641243407079</v>
+        <v>0.99730422320290779</v>
       </c>
       <c r="AP11">
-        <v>23.349105375368897</v>
+        <v>49.422574613357185</v>
       </c>
       <c r="AR11" t="s">
         <v>214</v>
@@ -6228,16 +6228,16 @@
         <v>219</v>
       </c>
       <c r="Y12" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="Z12" t="s">
         <v>260</v>
       </c>
       <c r="AA12">
-        <v>0.99606480786442353</v>
+        <v>0.99658775492800411</v>
       </c>
       <c r="AB12">
-        <v>72.145189152235062</v>
+        <v>62.557826319923819</v>
       </c>
       <c r="AD12" t="s">
         <v>214</v>
@@ -6270,10 +6270,10 @@
         <v>322</v>
       </c>
       <c r="AO12">
-        <v>0.99776911581804295</v>
+        <v>0.99805709209211746</v>
       </c>
       <c r="AP12">
-        <v>40.899543335879912</v>
+        <v>35.619978311179104</v>
       </c>
       <c r="AR12" t="s">
         <v>214</v>
@@ -6374,16 +6374,16 @@
         <v>221</v>
       </c>
       <c r="Y13" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="Z13" t="s">
         <v>261</v>
       </c>
       <c r="AA13">
-        <v>0.99785589517057005</v>
+        <v>0.99510886326373238</v>
       </c>
       <c r="AB13">
-        <v>39.308588539549028</v>
+        <v>89.670840164906522</v>
       </c>
       <c r="AD13" t="s">
         <v>214</v>
@@ -6416,10 +6416,10 @@
         <v>324</v>
       </c>
       <c r="AO13">
-        <v>0.99653588726932718</v>
+        <v>0.99622969699231045</v>
       </c>
       <c r="AP13">
-        <v>63.508733395668145</v>
+        <v>69.122221807641537</v>
       </c>
       <c r="AR13" t="s">
         <v>214</v>
@@ -6449,13 +6449,13 @@
         <v>382</v>
       </c>
       <c r="BB13" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="BC13">
-        <v>0.99353721168226494</v>
+        <v>0.99608994650263638</v>
       </c>
       <c r="BD13">
-        <v>780.55486105754892</v>
+        <v>589.950661136485</v>
       </c>
     </row>
     <row r="14" spans="2:56">
@@ -6562,10 +6562,10 @@
         <v>326</v>
       </c>
       <c r="AO14">
-        <v>0.9963019969989696</v>
+        <v>0.99827231256984739</v>
       </c>
       <c r="AP14">
-        <v>67.796721685557472</v>
+        <v>31.674269552798414</v>
       </c>
       <c r="AR14" t="s">
         <v>214</v>
@@ -6592,16 +6592,16 @@
         <v>364</v>
       </c>
       <c r="BA14" t="s">
+        <v>383</v>
+      </c>
+      <c r="BB14" t="s">
         <v>384</v>
       </c>
-      <c r="BB14" t="s">
-        <v>385</v>
-      </c>
       <c r="BC14">
-        <v>0.99615739524125424</v>
+        <v>0.99399682431672776</v>
       </c>
       <c r="BD14">
-        <v>584.91448865302027</v>
+        <v>746.2371176843244</v>
       </c>
     </row>
     <row r="15" spans="2:56">
@@ -6708,10 +6708,10 @@
         <v>328</v>
       </c>
       <c r="AO15">
-        <v>0.99622969699231045</v>
+        <v>0.99635146162488653</v>
       </c>
       <c r="AP15">
-        <v>69.122221807641537</v>
+        <v>66.889870210414614</v>
       </c>
       <c r="AR15" t="s">
         <v>214</v>
@@ -6738,10 +6738,10 @@
         <v>366</v>
       </c>
       <c r="BA15" t="s">
+        <v>385</v>
+      </c>
+      <c r="BB15" t="s">
         <v>386</v>
-      </c>
-      <c r="BB15" t="s">
-        <v>387</v>
       </c>
       <c r="BC15">
         <v>0.99255663966463281</v>
@@ -6851,13 +6851,13 @@
         <v>329</v>
       </c>
       <c r="AN16" t="s">
-        <v>330</v>
+        <v>268</v>
       </c>
       <c r="AO16">
-        <v>0.99802303154782224</v>
+        <v>0.99586212495478665</v>
       </c>
       <c r="AP16">
-        <v>36.244421623259619</v>
+        <v>75.861042495577635</v>
       </c>
       <c r="AR16" t="s">
         <v>214</v>
@@ -6884,16 +6884,16 @@
         <v>368</v>
       </c>
       <c r="BA16" t="s">
+        <v>387</v>
+      </c>
+      <c r="BB16" t="s">
         <v>388</v>
       </c>
-      <c r="BB16" t="s">
-        <v>381</v>
-      </c>
       <c r="BC16">
-        <v>0.99608994650263638</v>
+        <v>0.99615739524125424</v>
       </c>
       <c r="BD16">
-        <v>589.950661136485</v>
+        <v>584.91448865302027</v>
       </c>
     </row>
     <row r="17" spans="2:56">
@@ -6958,16 +6958,16 @@
         <v>229</v>
       </c>
       <c r="Y17" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="Z17" t="s">
         <v>265</v>
       </c>
       <c r="AA17">
-        <v>0.99481478101166732</v>
+        <v>0.99930490342600053</v>
       </c>
       <c r="AB17">
-        <v>95.062348119433295</v>
+        <v>12.743437189989784</v>
       </c>
       <c r="AD17" t="s">
         <v>214</v>
@@ -6994,16 +6994,16 @@
         <v>291</v>
       </c>
       <c r="AM17" t="s">
+        <v>330</v>
+      </c>
+      <c r="AN17" t="s">
         <v>331</v>
       </c>
-      <c r="AN17" t="s">
-        <v>332</v>
-      </c>
       <c r="AO17">
-        <v>0.99714358927215652</v>
+        <v>0.99749126227646956</v>
       </c>
       <c r="AP17">
-        <v>52.367530010463909</v>
+        <v>45.993524931390482</v>
       </c>
       <c r="AR17" t="s">
         <v>214</v>
@@ -7036,10 +7036,10 @@
         <v>390</v>
       </c>
       <c r="BC17">
-        <v>0.99399682431672776</v>
+        <v>0.99353721168226494</v>
       </c>
       <c r="BD17">
-        <v>746.2371176843244</v>
+        <v>780.55486105754892</v>
       </c>
     </row>
     <row r="18" spans="2:56">
@@ -7104,16 +7104,16 @@
         <v>231</v>
       </c>
       <c r="Y18" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="Z18" t="s">
         <v>266</v>
       </c>
       <c r="AA18">
-        <v>0.99681878296180493</v>
+        <v>0.99881801309037566</v>
       </c>
       <c r="AB18">
-        <v>58.322312366909152</v>
+        <v>21.669760009780138</v>
       </c>
       <c r="AD18" t="s">
         <v>214</v>
@@ -7140,16 +7140,16 @@
         <v>293</v>
       </c>
       <c r="AM18" t="s">
+        <v>332</v>
+      </c>
+      <c r="AN18" t="s">
         <v>333</v>
       </c>
-      <c r="AN18" t="s">
-        <v>334</v>
-      </c>
       <c r="AO18">
-        <v>0.99749126227646956</v>
+        <v>0.99807543246352515</v>
       </c>
       <c r="AP18">
-        <v>45.993524931390482</v>
+        <v>35.283738168705199</v>
       </c>
       <c r="AR18" t="s">
         <v>214</v>
@@ -7179,13 +7179,13 @@
         <v>391</v>
       </c>
       <c r="BB18" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="BC18">
-        <v>0.99564787435456037</v>
+        <v>0.99328660064428831</v>
       </c>
       <c r="BD18">
-        <v>622.95871485949408</v>
+        <v>799.26715189313825</v>
       </c>
     </row>
     <row r="19" spans="2:56">
@@ -7250,16 +7250,16 @@
         <v>233</v>
       </c>
       <c r="Y19" t="s">
-        <v>195</v>
+        <v>206</v>
       </c>
       <c r="Z19" t="s">
         <v>267</v>
       </c>
       <c r="AA19">
-        <v>0.99770934816564383</v>
+        <v>0.99790408176624201</v>
       </c>
       <c r="AB19">
-        <v>41.995283629862939</v>
+        <v>38.425167618896296</v>
       </c>
       <c r="AD19" t="s">
         <v>214</v>
@@ -7286,16 +7286,16 @@
         <v>295</v>
       </c>
       <c r="AM19" t="s">
+        <v>334</v>
+      </c>
+      <c r="AN19" t="s">
         <v>335</v>
       </c>
-      <c r="AN19" t="s">
-        <v>336</v>
-      </c>
       <c r="AO19">
-        <v>0.99807543246352515</v>
+        <v>0.99872641243407079</v>
       </c>
       <c r="AP19">
-        <v>35.283738168705199</v>
+        <v>23.349105375368897</v>
       </c>
       <c r="AR19" t="s">
         <v>214</v>
@@ -7322,16 +7322,16 @@
         <v>374</v>
       </c>
       <c r="BA19" t="s">
+        <v>392</v>
+      </c>
+      <c r="BB19" t="s">
         <v>393</v>
       </c>
-      <c r="BB19" t="s">
-        <v>385</v>
-      </c>
       <c r="BC19">
-        <v>0.99328660064428831</v>
+        <v>0.99644441082752833</v>
       </c>
       <c r="BD19">
-        <v>799.26715189313825</v>
+        <v>563.48399154455342</v>
       </c>
     </row>
     <row r="20" spans="2:56">
@@ -7396,16 +7396,16 @@
         <v>235</v>
       </c>
       <c r="Y20" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="Z20" t="s">
         <v>268</v>
       </c>
       <c r="AA20">
-        <v>0.9970292559096442</v>
+        <v>0.99606480786442353</v>
       </c>
       <c r="AB20">
-        <v>54.463641656523762</v>
+        <v>72.145189152235062</v>
       </c>
       <c r="AD20" t="s">
         <v>214</v>
@@ -7432,16 +7432,16 @@
         <v>297</v>
       </c>
       <c r="AM20" t="s">
+        <v>336</v>
+      </c>
+      <c r="AN20" t="s">
         <v>337</v>
       </c>
-      <c r="AN20" t="s">
-        <v>338</v>
-      </c>
       <c r="AO20">
-        <v>0.99845791964146047</v>
+        <v>0.99776911581804295</v>
       </c>
       <c r="AP20">
-        <v>28.2714732398913</v>
+        <v>40.899543335879912</v>
       </c>
       <c r="AR20" t="s">
         <v>214</v>
@@ -7471,13 +7471,13 @@
         <v>394</v>
       </c>
       <c r="BB20" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="BC20">
-        <v>0.99644441082752833</v>
+        <v>0.99564787435456037</v>
       </c>
       <c r="BD20">
-        <v>563.48399154455342</v>
+        <v>622.95871485949408</v>
       </c>
     </row>
     <row r="21" spans="2:56">
@@ -7542,16 +7542,16 @@
         <v>237</v>
       </c>
       <c r="Y21" t="s">
-        <v>208</v>
+        <v>193</v>
       </c>
       <c r="Z21" t="s">
         <v>269</v>
       </c>
       <c r="AA21">
-        <v>0.9982126095160021</v>
+        <v>0.99707401400885998</v>
       </c>
       <c r="AB21">
-        <v>32.768825539961391</v>
+        <v>53.643076504234422</v>
       </c>
       <c r="AD21" t="s">
         <v>214</v>
@@ -7578,16 +7578,16 @@
         <v>299</v>
       </c>
       <c r="AM21" t="s">
+        <v>338</v>
+      </c>
+      <c r="AN21" t="s">
         <v>339</v>
       </c>
-      <c r="AN21" t="s">
-        <v>340</v>
-      </c>
       <c r="AO21">
-        <v>0.99641308487583879</v>
+        <v>0.99653588726932718</v>
       </c>
       <c r="AP21">
-        <v>65.760110609622657</v>
+        <v>63.508733395668145</v>
       </c>
     </row>
     <row r="22" spans="2:56">
@@ -7652,16 +7652,16 @@
         <v>239</v>
       </c>
       <c r="Y22" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="Z22" t="s">
         <v>270</v>
       </c>
       <c r="AA22">
-        <v>0.99658775492800411</v>
+        <v>0.99826037700975512</v>
       </c>
       <c r="AB22">
-        <v>62.557826319923819</v>
+        <v>31.893088154488542</v>
       </c>
       <c r="AD22" t="s">
         <v>214</v>
@@ -7688,16 +7688,16 @@
         <v>301</v>
       </c>
       <c r="AM22" t="s">
+        <v>340</v>
+      </c>
+      <c r="AN22" t="s">
         <v>341</v>
       </c>
-      <c r="AN22" t="s">
-        <v>342</v>
-      </c>
       <c r="AO22">
-        <v>0.99449756685866841</v>
+        <v>0.99802303154782224</v>
       </c>
       <c r="AP22">
-        <v>100.87794092441324</v>
+        <v>36.244421623259619</v>
       </c>
     </row>
     <row r="23" spans="2:56">
@@ -7762,16 +7762,16 @@
         <v>241</v>
       </c>
       <c r="Y23" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="Z23" t="s">
         <v>271</v>
       </c>
       <c r="AA23">
-        <v>0.99510886326373238</v>
+        <v>0.99922515067657613</v>
       </c>
       <c r="AB23">
-        <v>89.670840164906522</v>
+        <v>14.205570929438155</v>
       </c>
       <c r="AD23" t="s">
         <v>214</v>
@@ -7798,16 +7798,16 @@
         <v>303</v>
       </c>
       <c r="AM23" t="s">
+        <v>342</v>
+      </c>
+      <c r="AN23" t="s">
         <v>343</v>
       </c>
-      <c r="AN23" t="s">
-        <v>344</v>
-      </c>
       <c r="AO23">
-        <v>0.99883902037019667</v>
+        <v>0.99714358927215652</v>
       </c>
       <c r="AP23">
-        <v>21.284626546395259</v>
+        <v>52.367530010463909</v>
       </c>
     </row>
     <row r="24" spans="2:56">
@@ -7872,16 +7872,16 @@
         <v>243</v>
       </c>
       <c r="Y24" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="Z24" t="s">
         <v>272</v>
       </c>
       <c r="AA24">
-        <v>0.99707401400885998</v>
+        <v>0.99770934816564383</v>
       </c>
       <c r="AB24">
-        <v>53.643076504234422</v>
+        <v>41.995283629862939</v>
       </c>
       <c r="AD24" t="s">
         <v>214</v>
@@ -7908,16 +7908,16 @@
         <v>305</v>
       </c>
       <c r="AM24" t="s">
+        <v>344</v>
+      </c>
+      <c r="AN24" t="s">
         <v>345</v>
       </c>
-      <c r="AN24" t="s">
-        <v>346</v>
-      </c>
       <c r="AO24">
-        <v>0.99521984547821263</v>
+        <v>0.9963019969989696</v>
       </c>
       <c r="AP24">
-        <v>87.636166232768815</v>
+        <v>67.796721685557472</v>
       </c>
     </row>
     <row r="25" spans="2:56">
@@ -7982,16 +7982,16 @@
         <v>245</v>
       </c>
       <c r="Y25" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="Z25" t="s">
         <v>273</v>
       </c>
       <c r="AA25">
-        <v>0.99826037700975512</v>
+        <v>0.9970292559096442</v>
       </c>
       <c r="AB25">
-        <v>31.893088154488542</v>
+        <v>54.463641656523762</v>
       </c>
       <c r="AD25" t="s">
         <v>214</v>
@@ -8018,16 +8018,16 @@
         <v>307</v>
       </c>
       <c r="AM25" t="s">
+        <v>346</v>
+      </c>
+      <c r="AN25" t="s">
         <v>347</v>
       </c>
-      <c r="AN25" t="s">
-        <v>348</v>
-      </c>
       <c r="AO25">
-        <v>0.99730422320290779</v>
+        <v>0.99845791964146047</v>
       </c>
       <c r="AP25">
-        <v>49.422574613357185</v>
+        <v>28.2714732398913</v>
       </c>
     </row>
     <row r="26" spans="2:56">
@@ -8092,16 +8092,16 @@
         <v>247</v>
       </c>
       <c r="Y26" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="Z26" t="s">
         <v>274</v>
       </c>
       <c r="AA26">
-        <v>0.99922515067657613</v>
+        <v>0.9982126095160021</v>
       </c>
       <c r="AB26">
-        <v>14.205570929438155</v>
+        <v>32.768825539961391</v>
       </c>
       <c r="AD26" t="s">
         <v>214</v>
@@ -8128,16 +8128,16 @@
         <v>309</v>
       </c>
       <c r="AM26" t="s">
+        <v>348</v>
+      </c>
+      <c r="AN26" t="s">
         <v>349</v>
       </c>
-      <c r="AN26" t="s">
-        <v>350</v>
-      </c>
       <c r="AO26">
-        <v>0.99805709209211746</v>
+        <v>0.99641308487583879</v>
       </c>
       <c r="AP26">
-        <v>35.619978311179104</v>
+        <v>65.760110609622657</v>
       </c>
     </row>
     <row r="27" spans="2:56">
@@ -8202,16 +8202,16 @@
         <v>249</v>
       </c>
       <c r="Y27" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="Z27" t="s">
         <v>275</v>
       </c>
       <c r="AA27">
-        <v>0.99730738889353909</v>
+        <v>0.99785589517057005</v>
       </c>
       <c r="AB27">
-        <v>49.364536951784054</v>
+        <v>39.308588539549028</v>
       </c>
       <c r="AD27" t="s">
         <v>214</v>
@@ -8238,16 +8238,16 @@
         <v>311</v>
       </c>
       <c r="AM27" t="s">
+        <v>350</v>
+      </c>
+      <c r="AN27" t="s">
         <v>351</v>
       </c>
-      <c r="AN27" t="s">
-        <v>352</v>
-      </c>
       <c r="AO27">
-        <v>0.99827231256984739</v>
+        <v>0.99449756685866841</v>
       </c>
       <c r="AP27">
-        <v>31.674269552798414</v>
+        <v>100.87794092441324</v>
       </c>
     </row>
     <row r="28" spans="2:56">
@@ -8312,16 +8312,16 @@
         <v>251</v>
       </c>
       <c r="Y28" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="Z28" t="s">
         <v>276</v>
       </c>
       <c r="AA28">
-        <v>0.99790408176624201</v>
+        <v>0.99481478101166732</v>
       </c>
       <c r="AB28">
-        <v>38.425167618896296</v>
+        <v>95.062348119433295</v>
       </c>
       <c r="AD28" t="s">
         <v>214</v>
@@ -8348,16 +8348,16 @@
         <v>313</v>
       </c>
       <c r="AM28" t="s">
+        <v>352</v>
+      </c>
+      <c r="AN28" t="s">
         <v>353</v>
       </c>
-      <c r="AN28" t="s">
-        <v>354</v>
-      </c>
       <c r="AO28">
-        <v>0.99635146162488653</v>
+        <v>0.99883902037019667</v>
       </c>
       <c r="AP28">
-        <v>66.889870210414614</v>
+        <v>21.284626546395259</v>
       </c>
     </row>
     <row r="29" spans="2:56">
@@ -8422,16 +8422,16 @@
         <v>253</v>
       </c>
       <c r="Y29" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="Z29" t="s">
         <v>277</v>
       </c>
       <c r="AA29">
-        <v>0.99930490342600053</v>
+        <v>0.99681878296180493</v>
       </c>
       <c r="AB29">
-        <v>12.743437189989784</v>
+        <v>58.322312366909152</v>
       </c>
       <c r="AD29" t="s">
         <v>214</v>
@@ -8458,16 +8458,16 @@
         <v>315</v>
       </c>
       <c r="AM29" t="s">
+        <v>354</v>
+      </c>
+      <c r="AN29" t="s">
         <v>355</v>
       </c>
-      <c r="AN29" t="s">
-        <v>260</v>
-      </c>
       <c r="AO29">
-        <v>0.99586212495478665</v>
+        <v>0.99521984547821263</v>
       </c>
       <c r="AP29">
-        <v>75.861042495577635</v>
+        <v>87.636166232768815</v>
       </c>
     </row>
     <row r="30" spans="2:56">
@@ -8532,16 +8532,16 @@
         <v>255</v>
       </c>
       <c r="Y30" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="Z30" t="s">
         <v>278</v>
       </c>
       <c r="AA30">
-        <v>0.99881801309037566</v>
+        <v>0.99693515631487983</v>
       </c>
       <c r="AB30">
-        <v>21.669760009780138</v>
+        <v>56.188800893869058</v>
       </c>
       <c r="AD30" t="s">
         <v>214</v>
@@ -8586,7 +8586,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59151317-8DD6-4792-A37C-CEF8C67A62EE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19FD8E05-430E-4DA8-9DE8-20D898A6DE14}">
   <dimension ref="B9:Z30"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8731,7 +8731,7 @@
         <v>435</v>
       </c>
       <c r="X11" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="Y11">
         <v>0.83925000000000005</v>
@@ -8766,7 +8766,7 @@
         <v>397</v>
       </c>
       <c r="K12" t="s">
-        <v>337</v>
+        <v>346</v>
       </c>
       <c r="L12">
         <v>0.42035497786033621</v>
@@ -8799,7 +8799,7 @@
         <v>437</v>
       </c>
       <c r="X12" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="Y12">
         <v>16.887</v>
@@ -8834,7 +8834,7 @@
         <v>399</v>
       </c>
       <c r="K13" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="L13">
         <v>1.6077871713950227</v>
@@ -8867,7 +8867,7 @@
         <v>439</v>
       </c>
       <c r="X13" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="Y13">
         <v>11.2965</v>
@@ -8902,7 +8902,7 @@
         <v>401</v>
       </c>
       <c r="K14" t="s">
-        <v>355</v>
+        <v>329</v>
       </c>
       <c r="L14">
         <v>2.531891424764753</v>
@@ -8935,7 +8935,7 @@
         <v>441</v>
       </c>
       <c r="X14" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="Y14">
         <v>6.6577500000000001</v>
@@ -8970,7 +8970,7 @@
         <v>403</v>
       </c>
       <c r="K15" t="s">
-        <v>325</v>
+        <v>344</v>
       </c>
       <c r="L15">
         <v>7.6497810049421515</v>
@@ -9003,7 +9003,7 @@
         <v>443</v>
       </c>
       <c r="X15" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="Y15">
         <v>17.089500000000001</v>
@@ -9038,7 +9038,7 @@
         <v>405</v>
       </c>
       <c r="K16" t="s">
-        <v>351</v>
+        <v>325</v>
       </c>
       <c r="L16">
         <v>0.60733325583919984</v>
@@ -9071,7 +9071,7 @@
         <v>445</v>
       </c>
       <c r="X16" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="Y16">
         <v>8.8230000000000004</v>
@@ -9106,7 +9106,7 @@
         <v>407</v>
       </c>
       <c r="K17" t="s">
-        <v>323</v>
+        <v>338</v>
       </c>
       <c r="L17">
         <v>0.78389041837100704</v>
@@ -9174,7 +9174,7 @@
         <v>409</v>
       </c>
       <c r="K18" t="s">
-        <v>345</v>
+        <v>354</v>
       </c>
       <c r="L18">
         <v>3.0365724666245324</v>
@@ -9242,7 +9242,7 @@
         <v>411</v>
       </c>
       <c r="K19" t="s">
-        <v>353</v>
+        <v>327</v>
       </c>
       <c r="L19">
         <v>0.22970161230087291</v>
@@ -9275,7 +9275,7 @@
         <v>451</v>
       </c>
       <c r="X19" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="Y19">
         <v>13.37175</v>
@@ -9310,7 +9310,7 @@
         <v>413</v>
       </c>
       <c r="K20" t="s">
-        <v>331</v>
+        <v>342</v>
       </c>
       <c r="L20">
         <v>0.27066515065379043</v>
@@ -9343,7 +9343,7 @@
         <v>453</v>
       </c>
       <c r="X20" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
       <c r="Y20">
         <v>3.9427500000000002</v>
@@ -9378,7 +9378,7 @@
         <v>415</v>
       </c>
       <c r="K21" t="s">
-        <v>329</v>
+        <v>340</v>
       </c>
       <c r="L21">
         <v>0.32193208719379746</v>
@@ -9413,7 +9413,7 @@
         <v>417</v>
       </c>
       <c r="K22" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="L22">
         <v>0.6573344927201471</v>
@@ -9448,7 +9448,7 @@
         <v>419</v>
       </c>
       <c r="K23" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
       <c r="L23">
         <v>0.28992997651770519</v>
@@ -9483,7 +9483,7 @@
         <v>421</v>
       </c>
       <c r="K24" t="s">
-        <v>347</v>
+        <v>319</v>
       </c>
       <c r="L24">
         <v>0.74609319967150689</v>
@@ -9518,7 +9518,7 @@
         <v>423</v>
       </c>
       <c r="K25" t="s">
-        <v>339</v>
+        <v>348</v>
       </c>
       <c r="L25">
         <v>0.35328950844501877</v>
@@ -9553,7 +9553,7 @@
         <v>425</v>
       </c>
       <c r="K26" t="s">
-        <v>341</v>
+        <v>350</v>
       </c>
       <c r="L26">
         <v>0.7924639655878376</v>
@@ -9588,7 +9588,7 @@
         <v>427</v>
       </c>
       <c r="K27" t="s">
-        <v>321</v>
+        <v>336</v>
       </c>
       <c r="L27">
         <v>0.55411362221124194</v>
@@ -9623,7 +9623,7 @@
         <v>429</v>
       </c>
       <c r="K28" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="L28">
         <v>1.4327274230737423</v>
@@ -9658,7 +9658,7 @@
         <v>431</v>
       </c>
       <c r="K29" t="s">
-        <v>319</v>
+        <v>334</v>
       </c>
       <c r="L29">
         <v>0.56742801517356967</v>
@@ -9693,7 +9693,7 @@
         <v>433</v>
       </c>
       <c r="K30" t="s">
-        <v>349</v>
+        <v>321</v>
       </c>
       <c r="L30">
         <v>0.35405891742987328</v>
@@ -9708,7 +9708,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{339FE14C-E19A-4BFE-A95A-E195613017B1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BEB3642-4757-487B-BE5B-3F7C2E0C5BED}">
   <dimension ref="B9:Y136"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14069,7 +14069,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B9325FF-5D1B-41D3-B3B3-572D34CFCA51}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A2659BC-18B1-4844-A6BC-86A7AC754AB2}">
   <dimension ref="B9:T88"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated POL_grids_kan50 model - 2026-09-06 18:29
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_POL_grids_kan50/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan50\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1593261B-018E-42A2-8374-FD8809C3FAAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED96CF02-0040-41D0-9880-EE0143F7B2E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -723,6 +723,42 @@
     <t>daynite</t>
   </si>
   <si>
+    <t>distr_solelc_spv_POL_003</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 3</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_007</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 7</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_016</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 16</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_014</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 14</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_008</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 8</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_004</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 4</t>
+  </si>
+  <si>
     <t>distr_solelc_spv_POL_006</t>
   </si>
   <si>
@@ -735,6 +771,18 @@
     <t>connecting solar to buses in cluster 10</t>
   </si>
   <si>
+    <t>distr_solelc_spv_POL_017</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 17</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_020</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 20</t>
+  </si>
+  <si>
     <t>distr_solelc_spv_POL_002</t>
   </si>
   <si>
@@ -753,22 +801,34 @@
     <t>connecting solar to buses in cluster 9</t>
   </si>
   <si>
-    <t>distr_solelc_spv_POL_017</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 17</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_020</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 20</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_014</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 14</t>
+    <t>distr_solelc_spv_POL_001</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 1</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_015</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 15</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_018</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 18</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_012</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 12</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_011</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 11</t>
   </si>
   <si>
     <t>distr_solelc_spv_POL_013</t>
@@ -777,66 +837,6 @@
     <t>connecting solar to buses in cluster 13</t>
   </si>
   <si>
-    <t>distr_solelc_spv_POL_001</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 1</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_015</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 15</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_018</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 18</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_003</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 3</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_007</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 7</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_016</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 16</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_004</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 4</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_012</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 12</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_011</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 11</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_008</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 8</t>
-  </si>
-  <si>
     <t>comm-in</t>
   </si>
   <si>
@@ -846,12 +846,36 @@
     <t>e_Lubin_POL,e_Poznan_POL,e_Koszalin_POL,e_Bydgoszcz_POL</t>
   </si>
   <si>
+    <t>e_Lubin_POL,e_Swidnica_POL,e_Wroclaw_POL,e_Poznan_POL,e_Olesnica_POL</t>
+  </si>
+  <si>
+    <t>e_Koszalin_POL,e_Ustka_POL,e_Slupsk_POL</t>
+  </si>
+  <si>
+    <t>e_Olesnica_POL,e_Konin_POL,e_PiotrkowTrybunalsk_POL,e_Plock_POL</t>
+  </si>
+  <si>
+    <t>e_BielskoBiala_POL,e_Katowice_POL,e_Krakow_POL,e_Tarnow_POL</t>
+  </si>
+  <si>
+    <t>e_Bydgoszcz_POL,e_Gdansk_POL,e_Grudziadz_POL,e_Kwidzyn_POL</t>
+  </si>
+  <si>
+    <t>e_GorzowWielkopolski_POL,e_Szczecin_POL,e_Police_POL</t>
+  </si>
+  <si>
     <t>e_Plock_POL,e_Olsztyn_POL,e_Warsaw_POL</t>
   </si>
   <si>
     <t>e_Elk_POL,e_Grajewo_POL</t>
   </si>
   <si>
+    <t>e_Konin_POL,e_Bydgoszcz_POL,e_Wloclawek_POL,e_Kwidzyn_POL,e_Plock_POL</t>
+  </si>
+  <si>
+    <t>e_OstrowiecSwietokrz_POL,e_Pulawy_POL,e_Warsaw_POL</t>
+  </si>
+  <si>
     <t>e_Legnica_POL,e_Swidnica_POL,e_KedzierzynKozle_POL,e_Opole_POL</t>
   </si>
   <si>
@@ -861,46 +885,94 @@
     <t>e_Pulawy_POL,e_Bialystok_POL,e_Chelm_POL</t>
   </si>
   <si>
-    <t>e_Konin_POL,e_Bydgoszcz_POL,e_Wloclawek_POL,e_Kwidzyn_POL,e_Plock_POL</t>
-  </si>
-  <si>
-    <t>e_OstrowiecSwietokrz_POL,e_Pulawy_POL,e_Warsaw_POL</t>
-  </si>
-  <si>
-    <t>e_BielskoBiala_POL,e_Katowice_POL,e_Krakow_POL,e_Tarnow_POL</t>
+    <t>e_Boleslawiec_POL,e_ZielonaGora_POL</t>
+  </si>
+  <si>
+    <t>e_Sosnowiec_POL,e_KedzierzynKozle_POL,e_Olesnica_POL,e_Gliwice_POL,e_Czestochowa_POL,e_Radomsko_POL,e_PiotrkowTrybunalsk_POL,e_Kielce_POL</t>
+  </si>
+  <si>
+    <t>e_Warsaw_POL,e_Lomza_POL</t>
+  </si>
+  <si>
+    <t>e_Krosno_POL,e_Mielec_POL,e_Debica_POL,e_Zamosc_POL</t>
+  </si>
+  <si>
+    <t>e_Lomza_POL,e_Elk_POL,e_Bialystok_POL,e_Grajewo_POL</t>
   </si>
   <si>
     <t>e_Rzeszow_POL,e_Zamosc_POL,e_Pulawy_POL,e_Chelm_POL</t>
   </si>
   <si>
-    <t>e_Boleslawiec_POL,e_ZielonaGora_POL</t>
-  </si>
-  <si>
-    <t>e_Sosnowiec_POL,e_KedzierzynKozle_POL,e_Olesnica_POL,e_Gliwice_POL,e_Czestochowa_POL,e_Radomsko_POL,e_PiotrkowTrybunalsk_POL,e_Kielce_POL</t>
-  </si>
-  <si>
-    <t>e_Warsaw_POL,e_Lomza_POL</t>
-  </si>
-  <si>
-    <t>e_Lubin_POL,e_Swidnica_POL,e_Wroclaw_POL,e_Poznan_POL,e_Olesnica_POL</t>
-  </si>
-  <si>
-    <t>e_Koszalin_POL,e_Ustka_POL,e_Slupsk_POL</t>
-  </si>
-  <si>
-    <t>e_Olesnica_POL,e_Konin_POL,e_PiotrkowTrybunalsk_POL,e_Plock_POL</t>
-  </si>
-  <si>
-    <t>e_GorzowWielkopolski_POL,e_Szczecin_POL,e_Police_POL</t>
-  </si>
-  <si>
-    <t>e_Krosno_POL,e_Mielec_POL,e_Debica_POL,e_Zamosc_POL</t>
-  </si>
-  <si>
-    <t>e_Lomza_POL,e_Elk_POL,e_Bialystok_POL,e_Grajewo_POL</t>
-  </si>
-  <si>
-    <t>e_Bydgoszcz_POL,e_Gdansk_POL,e_Grudziadz_POL,e_Kwidzyn_POL</t>
+    <t>distr_wonelc_won_POL_005</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 5</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_018</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 18</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_019</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 19</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_017</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 17</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_007</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 7</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_006</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 6</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_009</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 9</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_004</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 4</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_015</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 15</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_016</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 16</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_001</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 1</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_002</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 2</t>
   </si>
   <si>
     <t>distr_wonelc_won_POL_014</t>
@@ -915,28 +987,28 @@
     <t>connecting wind onshore to buses in cluster 20</t>
   </si>
   <si>
-    <t>distr_wonelc_won_POL_018</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 18</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_006</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 6</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_009</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 9</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_004</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 4</t>
+    <t>distr_wonelc_won_POL_013</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 13</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_008</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 8</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_011</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 11</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_010</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 10</t>
   </si>
   <si>
     <t>distr_wonelc_won_POL_012</t>
@@ -951,76 +1023,73 @@
     <t>connecting wind onshore to buses in cluster 3</t>
   </si>
   <si>
-    <t>distr_wonelc_won_POL_019</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 19</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_017</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 17</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_007</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 7</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_011</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 11</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_010</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 10</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_005</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 5</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_002</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 2</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_015</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 15</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_016</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 16</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_013</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 13</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_008</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 8</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_001</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 1</t>
+    <t>elc_won_POL_005</t>
+  </si>
+  <si>
+    <t>e_Lomza_POL,e_Elk_POL,e_Grajewo_POL,e_Bialystok_POL,e_Chelm_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_018</t>
+  </si>
+  <si>
+    <t>e_Boleslawiec_POL,e_Legnica_POL,e_Swidnica_POL,e_KedzierzynKozle_POL,e_Opole_POL,e_Olesnica_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_019</t>
+  </si>
+  <si>
+    <t>e_Katowice_POL,e_Czestochowa_POL,e_Krakow_POL,e_Kielce_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_017</t>
+  </si>
+  <si>
+    <t>e_Tarnow_POL,e_Krosno_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_007</t>
+  </si>
+  <si>
+    <t>e_Warsaw_POL,e_Plock_POL,e_Olsztyn_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_006</t>
+  </si>
+  <si>
+    <t>e_Olesnica_POL,e_Konin_POL,e_Bydgoszcz_POL,e_Wloclawek_POL,e_Kwidzyn_POL,e_Plock_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_009</t>
+  </si>
+  <si>
+    <t>e_Gdansk_POL,e_Grudziadz_POL,e_Kwidzyn_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_004</t>
+  </si>
+  <si>
+    <t>elc_won_POL_015</t>
+  </si>
+  <si>
+    <t>e_BielskoBiala_POL,e_Krakow_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_016</t>
+  </si>
+  <si>
+    <t>e_Krosno_POL,e_Debica_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_001</t>
+  </si>
+  <si>
+    <t>e_PiotrkowTrybunalsk_POL,e_Kielce_POL,e_Warsaw_POL,e_OstrowiecSwietokrz_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_002</t>
+  </si>
+  <si>
+    <t>e_Tarnow_POL,e_Kielce_POL,e_OstrowiecSwietokrz_POL,e_Mielec_POL,e_Pulawy_POL,e_Rzeszow_POL</t>
   </si>
   <si>
     <t>elc_won_POL_014</t>
@@ -1035,25 +1104,28 @@
     <t>e_Sosnowiec_POL,e_KedzierzynKozle_POL,e_Olesnica_POL,e_Gliwice_POL,e_Czestochowa_POL,e_Radomsko_POL</t>
   </si>
   <si>
-    <t>elc_won_POL_018</t>
-  </si>
-  <si>
-    <t>e_Boleslawiec_POL,e_Legnica_POL,e_Swidnica_POL,e_KedzierzynKozle_POL,e_Opole_POL,e_Olesnica_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_006</t>
-  </si>
-  <si>
-    <t>e_Olesnica_POL,e_Konin_POL,e_Bydgoszcz_POL,e_Wloclawek_POL,e_Kwidzyn_POL,e_Plock_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_009</t>
-  </si>
-  <si>
-    <t>e_Gdansk_POL,e_Grudziadz_POL,e_Kwidzyn_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_004</t>
+    <t>elc_won_POL_013</t>
+  </si>
+  <si>
+    <t>e_Lubin_POL,e_Wroclaw_POL,e_Poznan_POL,e_Olesnica_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_008</t>
+  </si>
+  <si>
+    <t>e_Olsztyn_POL,e_Elk_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_011</t>
+  </si>
+  <si>
+    <t>e_Boleslawiec_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_010</t>
+  </si>
+  <si>
+    <t>e_Police_POL,e_Koszalin_POL,e_Poznan_POL,e_Ustka_POL,e_Bydgoszcz_POL,e_Slupsk_POL,e_Gdansk_POL</t>
   </si>
   <si>
     <t>elc_won_POL_012</t>
@@ -1068,76 +1140,34 @@
     <t>e_Warsaw_POL,e_Lomza_POL,e_Pulawy_POL,e_Bialystok_POL</t>
   </si>
   <si>
-    <t>elc_won_POL_019</t>
-  </si>
-  <si>
-    <t>e_Katowice_POL,e_Czestochowa_POL,e_Krakow_POL,e_Kielce_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_017</t>
-  </si>
-  <si>
-    <t>e_Tarnow_POL,e_Krosno_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_007</t>
-  </si>
-  <si>
-    <t>e_Warsaw_POL,e_Plock_POL,e_Olsztyn_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_011</t>
-  </si>
-  <si>
-    <t>e_Boleslawiec_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_010</t>
-  </si>
-  <si>
-    <t>e_Police_POL,e_Koszalin_POL,e_Poznan_POL,e_Ustka_POL,e_Bydgoszcz_POL,e_Slupsk_POL,e_Gdansk_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_005</t>
-  </si>
-  <si>
-    <t>e_Lomza_POL,e_Elk_POL,e_Grajewo_POL,e_Bialystok_POL,e_Chelm_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_002</t>
-  </si>
-  <si>
-    <t>e_Tarnow_POL,e_Kielce_POL,e_OstrowiecSwietokrz_POL,e_Mielec_POL,e_Pulawy_POL,e_Rzeszow_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_015</t>
-  </si>
-  <si>
-    <t>e_BielskoBiala_POL,e_Krakow_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_016</t>
-  </si>
-  <si>
-    <t>e_Krosno_POL,e_Debica_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_013</t>
-  </si>
-  <si>
-    <t>e_Lubin_POL,e_Wroclaw_POL,e_Poznan_POL,e_Olesnica_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_008</t>
-  </si>
-  <si>
-    <t>e_Olsztyn_POL,e_Elk_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_001</t>
-  </si>
-  <si>
-    <t>e_PiotrkowTrybunalsk_POL,e_Kielce_POL,e_Warsaw_POL,e_OstrowiecSwietokrz_POL</t>
+    <t>distr_wofelc_wof_POL_002</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 2</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_POL_004</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 4</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_POL_006</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 6</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_POL_005</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 5</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_POL_001</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 1</t>
   </si>
   <si>
     <t>distr_wofelc_wof_POL_008</t>
@@ -1152,6 +1182,12 @@
     <t>connecting wind offshore to buses in cluster 7</t>
   </si>
   <si>
+    <t>distr_wofelc_wof_POL_003</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 3</t>
+  </si>
+  <si>
     <t>distr_wofelc_wof_POL_010</t>
   </si>
   <si>
@@ -1164,40 +1200,31 @@
     <t>connecting wind offshore to buses in cluster 9</t>
   </si>
   <si>
-    <t>distr_wofelc_wof_POL_004</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 4</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_POL_006</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 6</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_POL_002</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 2</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_POL_005</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 5</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_POL_001</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 1</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_POL_003</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 3</t>
+    <t>elc_wof_POL_002</t>
+  </si>
+  <si>
+    <t>e_Gdynia_POL,e_Gdansk_POL</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_004</t>
+  </si>
+  <si>
+    <t>e_Ustka_POL,e_Gdynia_POL</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_006</t>
+  </si>
+  <si>
+    <t>e_Gdynia_POL</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_005</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_001</t>
+  </si>
+  <si>
+    <t>e_Gdansk_POL</t>
   </si>
   <si>
     <t>elc_wof_POL_008</t>
@@ -1212,6 +1239,9 @@
     <t>e_Koszalin_POL</t>
   </si>
   <si>
+    <t>elc_wof_POL_003</t>
+  </si>
+  <si>
     <t>elc_wof_POL_010</t>
   </si>
   <si>
@@ -1219,36 +1249,6 @@
   </si>
   <si>
     <t>e_Koszalin_POL,e_Ustka_POL</t>
-  </si>
-  <si>
-    <t>elc_wof_POL_004</t>
-  </si>
-  <si>
-    <t>e_Ustka_POL,e_Gdynia_POL</t>
-  </si>
-  <si>
-    <t>elc_wof_POL_006</t>
-  </si>
-  <si>
-    <t>e_Gdynia_POL</t>
-  </si>
-  <si>
-    <t>elc_wof_POL_002</t>
-  </si>
-  <si>
-    <t>e_Gdynia_POL,e_Gdansk_POL</t>
-  </si>
-  <si>
-    <t>elc_wof_POL_005</t>
-  </si>
-  <si>
-    <t>elc_wof_POL_001</t>
-  </si>
-  <si>
-    <t>e_Gdansk_POL</t>
-  </si>
-  <si>
-    <t>elc_wof_POL_003</t>
   </si>
   <si>
     <t>e_won_POL_001</t>
@@ -5844,7 +5844,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0C0ECA9-2976-4949-BB23-4E467F422200}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{015DDA11-CC52-47AB-805C-AA4E40561873}">
   <dimension ref="B9:BD30"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6124,10 +6124,10 @@
         <v>320</v>
       </c>
       <c r="AO11">
-        <v>0.99730422320290779</v>
+        <v>0.9963019969989696</v>
       </c>
       <c r="AP11">
-        <v>49.422574613357185</v>
+        <v>67.796721685557472</v>
       </c>
       <c r="AR11" t="s">
         <v>214</v>
@@ -6160,10 +6160,10 @@
         <v>379</v>
       </c>
       <c r="BC11">
-        <v>0.99383352379209899</v>
+        <v>0.99353721168226494</v>
       </c>
       <c r="BD11">
-        <v>758.43022352327353</v>
+        <v>780.55486105754892</v>
       </c>
     </row>
     <row r="12" spans="2:56">
@@ -6228,16 +6228,16 @@
         <v>219</v>
       </c>
       <c r="Y12" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="Z12" t="s">
         <v>260</v>
       </c>
       <c r="AA12">
-        <v>0.99658775492800411</v>
+        <v>0.99770934816564383</v>
       </c>
       <c r="AB12">
-        <v>62.557826319923819</v>
+        <v>41.995283629862939</v>
       </c>
       <c r="AD12" t="s">
         <v>214</v>
@@ -6270,10 +6270,10 @@
         <v>322</v>
       </c>
       <c r="AO12">
-        <v>0.99805709209211746</v>
+        <v>0.99622969699231045</v>
       </c>
       <c r="AP12">
-        <v>35.619978311179104</v>
+        <v>69.122221807641537</v>
       </c>
       <c r="AR12" t="s">
         <v>214</v>
@@ -6306,10 +6306,10 @@
         <v>381</v>
       </c>
       <c r="BC12">
-        <v>0.99603306101923861</v>
+        <v>0.99255663966463281</v>
       </c>
       <c r="BD12">
-        <v>594.19811056351818</v>
+        <v>853.77090504074806</v>
       </c>
     </row>
     <row r="13" spans="2:56">
@@ -6374,16 +6374,16 @@
         <v>221</v>
       </c>
       <c r="Y13" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="Z13" t="s">
         <v>261</v>
       </c>
       <c r="AA13">
-        <v>0.99510886326373238</v>
+        <v>0.9970292559096442</v>
       </c>
       <c r="AB13">
-        <v>89.670840164906522</v>
+        <v>54.463641656523762</v>
       </c>
       <c r="AD13" t="s">
         <v>214</v>
@@ -6416,10 +6416,10 @@
         <v>324</v>
       </c>
       <c r="AO13">
-        <v>0.99622969699231045</v>
+        <v>0.99872641243407079</v>
       </c>
       <c r="AP13">
-        <v>69.122221807641537</v>
+        <v>23.349105375368897</v>
       </c>
       <c r="AR13" t="s">
         <v>214</v>
@@ -6449,13 +6449,13 @@
         <v>382</v>
       </c>
       <c r="BB13" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="BC13">
-        <v>0.99608994650263638</v>
+        <v>0.99615739524125424</v>
       </c>
       <c r="BD13">
-        <v>589.950661136485</v>
+        <v>584.91448865302027</v>
       </c>
     </row>
     <row r="14" spans="2:56">
@@ -6520,16 +6520,16 @@
         <v>223</v>
       </c>
       <c r="Y14" t="s">
-        <v>194</v>
+        <v>208</v>
       </c>
       <c r="Z14" t="s">
         <v>262</v>
       </c>
       <c r="AA14">
-        <v>0.99515616506526205</v>
+        <v>0.9982126095160021</v>
       </c>
       <c r="AB14">
-        <v>88.803640470195262</v>
+        <v>32.768825539961391</v>
       </c>
       <c r="AD14" t="s">
         <v>214</v>
@@ -6562,10 +6562,10 @@
         <v>326</v>
       </c>
       <c r="AO14">
-        <v>0.99827231256984739</v>
+        <v>0.99776911581804295</v>
       </c>
       <c r="AP14">
-        <v>31.674269552798414</v>
+        <v>40.899543335879912</v>
       </c>
       <c r="AR14" t="s">
         <v>214</v>
@@ -6592,16 +6592,16 @@
         <v>364</v>
       </c>
       <c r="BA14" t="s">
+        <v>384</v>
+      </c>
+      <c r="BB14" t="s">
         <v>383</v>
       </c>
-      <c r="BB14" t="s">
-        <v>384</v>
-      </c>
       <c r="BC14">
-        <v>0.99399682431672776</v>
+        <v>0.99328660064428831</v>
       </c>
       <c r="BD14">
-        <v>746.2371176843244</v>
+        <v>799.26715189313825</v>
       </c>
     </row>
     <row r="15" spans="2:56">
@@ -6666,16 +6666,16 @@
         <v>225</v>
       </c>
       <c r="Y15" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="Z15" t="s">
         <v>263</v>
       </c>
       <c r="AA15">
-        <v>0.99728872234103139</v>
+        <v>0.99790408176624201</v>
       </c>
       <c r="AB15">
-        <v>49.70675708109188</v>
+        <v>38.425167618896296</v>
       </c>
       <c r="AD15" t="s">
         <v>214</v>
@@ -6708,10 +6708,10 @@
         <v>328</v>
       </c>
       <c r="AO15">
-        <v>0.99635146162488653</v>
+        <v>0.99653588726932718</v>
       </c>
       <c r="AP15">
-        <v>66.889870210414614</v>
+        <v>63.508733395668145</v>
       </c>
       <c r="AR15" t="s">
         <v>214</v>
@@ -6744,10 +6744,10 @@
         <v>386</v>
       </c>
       <c r="BC15">
-        <v>0.99255663966463281</v>
+        <v>0.99644441082752833</v>
       </c>
       <c r="BD15">
-        <v>853.77090504074806</v>
+        <v>563.48399154455342</v>
       </c>
     </row>
     <row r="16" spans="2:56">
@@ -6812,16 +6812,16 @@
         <v>227</v>
       </c>
       <c r="Y16" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="Z16" t="s">
         <v>264</v>
       </c>
       <c r="AA16">
-        <v>0.99583567586599486</v>
+        <v>0.99693515631487983</v>
       </c>
       <c r="AB16">
-        <v>76.34594245676044</v>
+        <v>56.188800893869058</v>
       </c>
       <c r="AD16" t="s">
         <v>214</v>
@@ -6851,13 +6851,13 @@
         <v>329</v>
       </c>
       <c r="AN16" t="s">
-        <v>268</v>
+        <v>330</v>
       </c>
       <c r="AO16">
-        <v>0.99586212495478665</v>
+        <v>0.99827231256984739</v>
       </c>
       <c r="AP16">
-        <v>75.861042495577635</v>
+        <v>31.674269552798414</v>
       </c>
       <c r="AR16" t="s">
         <v>214</v>
@@ -6890,10 +6890,10 @@
         <v>388</v>
       </c>
       <c r="BC16">
-        <v>0.99615739524125424</v>
+        <v>0.99383352379209899</v>
       </c>
       <c r="BD16">
-        <v>584.91448865302027</v>
+        <v>758.43022352327353</v>
       </c>
     </row>
     <row r="17" spans="2:56">
@@ -6958,16 +6958,16 @@
         <v>229</v>
       </c>
       <c r="Y17" t="s">
-        <v>209</v>
+        <v>196</v>
       </c>
       <c r="Z17" t="s">
         <v>265</v>
       </c>
       <c r="AA17">
-        <v>0.99930490342600053</v>
+        <v>0.99785589517057005</v>
       </c>
       <c r="AB17">
-        <v>12.743437189989784</v>
+        <v>39.308588539549028</v>
       </c>
       <c r="AD17" t="s">
         <v>214</v>
@@ -6994,16 +6994,16 @@
         <v>291</v>
       </c>
       <c r="AM17" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="AN17" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="AO17">
-        <v>0.99749126227646956</v>
+        <v>0.99635146162488653</v>
       </c>
       <c r="AP17">
-        <v>45.993524931390482</v>
+        <v>66.889870210414614</v>
       </c>
       <c r="AR17" t="s">
         <v>214</v>
@@ -7036,10 +7036,10 @@
         <v>390</v>
       </c>
       <c r="BC17">
-        <v>0.99353721168226494</v>
+        <v>0.99603306101923861</v>
       </c>
       <c r="BD17">
-        <v>780.55486105754892</v>
+        <v>594.19811056351818</v>
       </c>
     </row>
     <row r="18" spans="2:56">
@@ -7104,16 +7104,16 @@
         <v>231</v>
       </c>
       <c r="Y18" t="s">
-        <v>212</v>
+        <v>198</v>
       </c>
       <c r="Z18" t="s">
         <v>266</v>
       </c>
       <c r="AA18">
-        <v>0.99881801309037566</v>
+        <v>0.99658775492800411</v>
       </c>
       <c r="AB18">
-        <v>21.669760009780138</v>
+        <v>62.557826319923819</v>
       </c>
       <c r="AD18" t="s">
         <v>214</v>
@@ -7140,16 +7140,16 @@
         <v>293</v>
       </c>
       <c r="AM18" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="AN18" t="s">
-        <v>333</v>
+        <v>278</v>
       </c>
       <c r="AO18">
-        <v>0.99807543246352515</v>
+        <v>0.99586212495478665</v>
       </c>
       <c r="AP18">
-        <v>35.283738168705199</v>
+        <v>75.861042495577635</v>
       </c>
       <c r="AR18" t="s">
         <v>214</v>
@@ -7179,13 +7179,13 @@
         <v>391</v>
       </c>
       <c r="BB18" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="BC18">
-        <v>0.99328660064428831</v>
+        <v>0.99564787435456037</v>
       </c>
       <c r="BD18">
-        <v>799.26715189313825</v>
+        <v>622.95871485949408</v>
       </c>
     </row>
     <row r="19" spans="2:56">
@@ -7250,16 +7250,16 @@
         <v>233</v>
       </c>
       <c r="Y19" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="Z19" t="s">
         <v>267</v>
       </c>
       <c r="AA19">
-        <v>0.99790408176624201</v>
+        <v>0.99510886326373238</v>
       </c>
       <c r="AB19">
-        <v>38.425167618896296</v>
+        <v>89.670840164906522</v>
       </c>
       <c r="AD19" t="s">
         <v>214</v>
@@ -7292,10 +7292,10 @@
         <v>335</v>
       </c>
       <c r="AO19">
-        <v>0.99872641243407079</v>
+        <v>0.99641308487583879</v>
       </c>
       <c r="AP19">
-        <v>23.349105375368897</v>
+        <v>65.760110609622657</v>
       </c>
       <c r="AR19" t="s">
         <v>214</v>
@@ -7325,13 +7325,13 @@
         <v>392</v>
       </c>
       <c r="BB19" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="BC19">
-        <v>0.99644441082752833</v>
+        <v>0.99608994650263638</v>
       </c>
       <c r="BD19">
-        <v>563.48399154455342</v>
+        <v>589.950661136485</v>
       </c>
     </row>
     <row r="20" spans="2:56">
@@ -7396,16 +7396,16 @@
         <v>235</v>
       </c>
       <c r="Y20" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="Z20" t="s">
         <v>268</v>
       </c>
       <c r="AA20">
-        <v>0.99606480786442353</v>
+        <v>0.99930490342600053</v>
       </c>
       <c r="AB20">
-        <v>72.145189152235062</v>
+        <v>12.743437189989784</v>
       </c>
       <c r="AD20" t="s">
         <v>214</v>
@@ -7438,10 +7438,10 @@
         <v>337</v>
       </c>
       <c r="AO20">
-        <v>0.99776911581804295</v>
+        <v>0.99449756685866841</v>
       </c>
       <c r="AP20">
-        <v>40.899543335879912</v>
+        <v>100.87794092441324</v>
       </c>
       <c r="AR20" t="s">
         <v>214</v>
@@ -7468,16 +7468,16 @@
         <v>376</v>
       </c>
       <c r="BA20" t="s">
+        <v>393</v>
+      </c>
+      <c r="BB20" t="s">
         <v>394</v>
       </c>
-      <c r="BB20" t="s">
-        <v>393</v>
-      </c>
       <c r="BC20">
-        <v>0.99564787435456037</v>
+        <v>0.99399682431672776</v>
       </c>
       <c r="BD20">
-        <v>622.95871485949408</v>
+        <v>746.2371176843244</v>
       </c>
     </row>
     <row r="21" spans="2:56">
@@ -7542,16 +7542,16 @@
         <v>237</v>
       </c>
       <c r="Y21" t="s">
-        <v>193</v>
+        <v>212</v>
       </c>
       <c r="Z21" t="s">
         <v>269</v>
       </c>
       <c r="AA21">
-        <v>0.99707401400885998</v>
+        <v>0.99881801309037566</v>
       </c>
       <c r="AB21">
-        <v>53.643076504234422</v>
+        <v>21.669760009780138</v>
       </c>
       <c r="AD21" t="s">
         <v>214</v>
@@ -7584,10 +7584,10 @@
         <v>339</v>
       </c>
       <c r="AO21">
-        <v>0.99653588726932718</v>
+        <v>0.99871360797890252</v>
       </c>
       <c r="AP21">
-        <v>63.508733395668145</v>
+        <v>23.583853720120768</v>
       </c>
     </row>
     <row r="22" spans="2:56">
@@ -7652,16 +7652,16 @@
         <v>239</v>
       </c>
       <c r="Y22" t="s">
-        <v>207</v>
+        <v>194</v>
       </c>
       <c r="Z22" t="s">
         <v>270</v>
       </c>
       <c r="AA22">
-        <v>0.99826037700975512</v>
+        <v>0.99515616506526205</v>
       </c>
       <c r="AB22">
-        <v>31.893088154488542</v>
+        <v>88.803640470195262</v>
       </c>
       <c r="AD22" t="s">
         <v>214</v>
@@ -7694,10 +7694,10 @@
         <v>341</v>
       </c>
       <c r="AO22">
-        <v>0.99802303154782224</v>
+        <v>0.99845791964146047</v>
       </c>
       <c r="AP22">
-        <v>36.244421623259619</v>
+        <v>28.2714732398913</v>
       </c>
     </row>
     <row r="23" spans="2:56">
@@ -7762,16 +7762,16 @@
         <v>241</v>
       </c>
       <c r="Y23" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="Z23" t="s">
         <v>271</v>
       </c>
       <c r="AA23">
-        <v>0.99922515067657613</v>
+        <v>0.99728872234103139</v>
       </c>
       <c r="AB23">
-        <v>14.205570929438155</v>
+        <v>49.70675708109188</v>
       </c>
       <c r="AD23" t="s">
         <v>214</v>
@@ -7804,10 +7804,10 @@
         <v>343</v>
       </c>
       <c r="AO23">
-        <v>0.99714358927215652</v>
+        <v>0.99730422320290779</v>
       </c>
       <c r="AP23">
-        <v>52.367530010463909</v>
+        <v>49.422574613357185</v>
       </c>
     </row>
     <row r="24" spans="2:56">
@@ -7872,16 +7872,16 @@
         <v>243</v>
       </c>
       <c r="Y24" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="Z24" t="s">
         <v>272</v>
       </c>
       <c r="AA24">
-        <v>0.99770934816564383</v>
+        <v>0.99583567586599486</v>
       </c>
       <c r="AB24">
-        <v>41.995283629862939</v>
+        <v>76.34594245676044</v>
       </c>
       <c r="AD24" t="s">
         <v>214</v>
@@ -7914,10 +7914,10 @@
         <v>345</v>
       </c>
       <c r="AO24">
-        <v>0.9963019969989696</v>
+        <v>0.99805709209211746</v>
       </c>
       <c r="AP24">
-        <v>67.796721685557472</v>
+        <v>35.619978311179104</v>
       </c>
     </row>
     <row r="25" spans="2:56">
@@ -7982,16 +7982,16 @@
         <v>245</v>
       </c>
       <c r="Y25" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="Z25" t="s">
         <v>273</v>
       </c>
       <c r="AA25">
-        <v>0.9970292559096442</v>
+        <v>0.99707401400885998</v>
       </c>
       <c r="AB25">
-        <v>54.463641656523762</v>
+        <v>53.643076504234422</v>
       </c>
       <c r="AD25" t="s">
         <v>214</v>
@@ -8024,10 +8024,10 @@
         <v>347</v>
       </c>
       <c r="AO25">
-        <v>0.99845791964146047</v>
+        <v>0.99883902037019667</v>
       </c>
       <c r="AP25">
-        <v>28.2714732398913</v>
+        <v>21.284626546395259</v>
       </c>
     </row>
     <row r="26" spans="2:56">
@@ -8092,16 +8092,16 @@
         <v>247</v>
       </c>
       <c r="Y26" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="Z26" t="s">
         <v>274</v>
       </c>
       <c r="AA26">
-        <v>0.9982126095160021</v>
+        <v>0.99826037700975512</v>
       </c>
       <c r="AB26">
-        <v>32.768825539961391</v>
+        <v>31.893088154488542</v>
       </c>
       <c r="AD26" t="s">
         <v>214</v>
@@ -8134,10 +8134,10 @@
         <v>349</v>
       </c>
       <c r="AO26">
-        <v>0.99641308487583879</v>
+        <v>0.99521984547821263</v>
       </c>
       <c r="AP26">
-        <v>65.760110609622657</v>
+        <v>87.636166232768815</v>
       </c>
     </row>
     <row r="27" spans="2:56">
@@ -8202,16 +8202,16 @@
         <v>249</v>
       </c>
       <c r="Y27" t="s">
-        <v>196</v>
+        <v>210</v>
       </c>
       <c r="Z27" t="s">
         <v>275</v>
       </c>
       <c r="AA27">
-        <v>0.99785589517057005</v>
+        <v>0.99922515067657613</v>
       </c>
       <c r="AB27">
-        <v>39.308588539549028</v>
+        <v>14.205570929438155</v>
       </c>
       <c r="AD27" t="s">
         <v>214</v>
@@ -8244,10 +8244,10 @@
         <v>351</v>
       </c>
       <c r="AO27">
-        <v>0.99449756685866841</v>
+        <v>0.99802303154782224</v>
       </c>
       <c r="AP27">
-        <v>100.87794092441324</v>
+        <v>36.244421623259619</v>
       </c>
     </row>
     <row r="28" spans="2:56">
@@ -8354,10 +8354,10 @@
         <v>353</v>
       </c>
       <c r="AO28">
-        <v>0.99883902037019667</v>
+        <v>0.99714358927215652</v>
       </c>
       <c r="AP28">
-        <v>21.284626546395259</v>
+        <v>52.367530010463909</v>
       </c>
     </row>
     <row r="29" spans="2:56">
@@ -8464,10 +8464,10 @@
         <v>355</v>
       </c>
       <c r="AO29">
-        <v>0.99521984547821263</v>
+        <v>0.99749126227646956</v>
       </c>
       <c r="AP29">
-        <v>87.636166232768815</v>
+        <v>45.993524931390482</v>
       </c>
     </row>
     <row r="30" spans="2:56">
@@ -8532,16 +8532,16 @@
         <v>255</v>
       </c>
       <c r="Y30" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="Z30" t="s">
         <v>278</v>
       </c>
       <c r="AA30">
-        <v>0.99693515631487983</v>
+        <v>0.99606480786442353</v>
       </c>
       <c r="AB30">
-        <v>56.188800893869058</v>
+        <v>72.145189152235062</v>
       </c>
       <c r="AD30" t="s">
         <v>214</v>
@@ -8574,10 +8574,10 @@
         <v>357</v>
       </c>
       <c r="AO30">
-        <v>0.99871360797890252</v>
+        <v>0.99807543246352515</v>
       </c>
       <c r="AP30">
-        <v>23.583853720120768</v>
+        <v>35.283738168705199</v>
       </c>
     </row>
   </sheetData>
@@ -8586,7 +8586,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19FD8E05-430E-4DA8-9DE8-20D898A6DE14}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4DE3BD5-D628-494D-886B-3AAD1B93E6F3}">
   <dimension ref="B9:Z30"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8698,7 +8698,7 @@
         <v>395</v>
       </c>
       <c r="K11" t="s">
-        <v>356</v>
+        <v>338</v>
       </c>
       <c r="L11">
         <v>0.30278350605008381</v>
@@ -8731,7 +8731,7 @@
         <v>435</v>
       </c>
       <c r="X11" t="s">
-        <v>392</v>
+        <v>385</v>
       </c>
       <c r="Y11">
         <v>0.83925000000000005</v>
@@ -8766,7 +8766,7 @@
         <v>397</v>
       </c>
       <c r="K12" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
       <c r="L12">
         <v>0.42035497786033621</v>
@@ -8799,7 +8799,7 @@
         <v>437</v>
       </c>
       <c r="X12" t="s">
-        <v>389</v>
+        <v>378</v>
       </c>
       <c r="Y12">
         <v>16.887</v>
@@ -8834,7 +8834,7 @@
         <v>399</v>
       </c>
       <c r="K13" t="s">
-        <v>332</v>
+        <v>356</v>
       </c>
       <c r="L13">
         <v>1.6077871713950227</v>
@@ -8867,7 +8867,7 @@
         <v>439</v>
       </c>
       <c r="X13" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="Y13">
         <v>11.2965</v>
@@ -8902,7 +8902,7 @@
         <v>401</v>
       </c>
       <c r="K14" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="L14">
         <v>2.531891424764753</v>
@@ -8935,7 +8935,7 @@
         <v>441</v>
       </c>
       <c r="X14" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="Y14">
         <v>6.6577500000000001</v>
@@ -8970,7 +8970,7 @@
         <v>403</v>
       </c>
       <c r="K15" t="s">
-        <v>344</v>
+        <v>319</v>
       </c>
       <c r="L15">
         <v>7.6497810049421515</v>
@@ -9003,7 +9003,7 @@
         <v>443</v>
       </c>
       <c r="X15" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="Y15">
         <v>17.089500000000001</v>
@@ -9038,7 +9038,7 @@
         <v>405</v>
       </c>
       <c r="K16" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="L16">
         <v>0.60733325583919984</v>
@@ -9071,7 +9071,7 @@
         <v>445</v>
       </c>
       <c r="X16" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="Y16">
         <v>8.8230000000000004</v>
@@ -9106,7 +9106,7 @@
         <v>407</v>
       </c>
       <c r="K17" t="s">
-        <v>338</v>
+        <v>327</v>
       </c>
       <c r="L17">
         <v>0.78389041837100704</v>
@@ -9139,7 +9139,7 @@
         <v>447</v>
       </c>
       <c r="X17" t="s">
-        <v>380</v>
+        <v>389</v>
       </c>
       <c r="Y17">
         <v>0.22650000000000001</v>
@@ -9174,7 +9174,7 @@
         <v>409</v>
       </c>
       <c r="K18" t="s">
-        <v>354</v>
+        <v>348</v>
       </c>
       <c r="L18">
         <v>3.0365724666245324</v>
@@ -9207,7 +9207,7 @@
         <v>449</v>
       </c>
       <c r="X18" t="s">
-        <v>378</v>
+        <v>387</v>
       </c>
       <c r="Y18">
         <v>9.5062499999999996</v>
@@ -9242,7 +9242,7 @@
         <v>411</v>
       </c>
       <c r="K19" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="L19">
         <v>0.22970161230087291</v>
@@ -9275,7 +9275,7 @@
         <v>451</v>
       </c>
       <c r="X19" t="s">
-        <v>383</v>
+        <v>393</v>
       </c>
       <c r="Y19">
         <v>13.37175</v>
@@ -9310,7 +9310,7 @@
         <v>413</v>
       </c>
       <c r="K20" t="s">
-        <v>342</v>
+        <v>352</v>
       </c>
       <c r="L20">
         <v>0.27066515065379043</v>
@@ -9343,7 +9343,7 @@
         <v>453</v>
       </c>
       <c r="X20" t="s">
-        <v>382</v>
+        <v>392</v>
       </c>
       <c r="Y20">
         <v>3.9427500000000002</v>
@@ -9378,7 +9378,7 @@
         <v>415</v>
       </c>
       <c r="K21" t="s">
-        <v>340</v>
+        <v>350</v>
       </c>
       <c r="L21">
         <v>0.32193208719379746</v>
@@ -9413,7 +9413,7 @@
         <v>417</v>
       </c>
       <c r="K22" t="s">
-        <v>330</v>
+        <v>354</v>
       </c>
       <c r="L22">
         <v>0.6573344927201471</v>
@@ -9448,7 +9448,7 @@
         <v>419</v>
       </c>
       <c r="K23" t="s">
-        <v>352</v>
+        <v>346</v>
       </c>
       <c r="L23">
         <v>0.28992997651770519</v>
@@ -9483,7 +9483,7 @@
         <v>421</v>
       </c>
       <c r="K24" t="s">
-        <v>319</v>
+        <v>342</v>
       </c>
       <c r="L24">
         <v>0.74609319967150689</v>
@@ -9518,7 +9518,7 @@
         <v>423</v>
       </c>
       <c r="K25" t="s">
-        <v>348</v>
+        <v>334</v>
       </c>
       <c r="L25">
         <v>0.35328950844501877</v>
@@ -9553,7 +9553,7 @@
         <v>425</v>
       </c>
       <c r="K26" t="s">
-        <v>350</v>
+        <v>336</v>
       </c>
       <c r="L26">
         <v>0.7924639655878376</v>
@@ -9588,7 +9588,7 @@
         <v>427</v>
       </c>
       <c r="K27" t="s">
-        <v>336</v>
+        <v>325</v>
       </c>
       <c r="L27">
         <v>0.55411362221124194</v>
@@ -9623,7 +9623,7 @@
         <v>429</v>
       </c>
       <c r="K28" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="L28">
         <v>1.4327274230737423</v>
@@ -9658,7 +9658,7 @@
         <v>431</v>
       </c>
       <c r="K29" t="s">
-        <v>334</v>
+        <v>323</v>
       </c>
       <c r="L29">
         <v>0.56742801517356967</v>
@@ -9693,7 +9693,7 @@
         <v>433</v>
       </c>
       <c r="K30" t="s">
-        <v>321</v>
+        <v>344</v>
       </c>
       <c r="L30">
         <v>0.35405891742987328</v>
@@ -9708,7 +9708,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BEB3642-4757-487B-BE5B-3F7C2E0C5BED}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50359684-D83D-45E3-9B6B-8FF18A0F48EC}">
   <dimension ref="B9:Y136"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14069,7 +14069,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A2659BC-18B1-4844-A6BC-86A7AC754AB2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7A9747E-B0EF-458E-A091-675018C9E90C}">
   <dimension ref="B9:T88"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>